<commit_message>
Aggiornamento file e calendario
</commit_message>
<xml_diff>
--- a/segreteria/Calendario esami LM.xlsx
+++ b/segreteria/Calendario esami LM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saint\unipavia\segreteria\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{380983EA-90B0-4596-9B68-73D0919A5128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73A6277E-F146-4E4B-AA75-B5C7152BAD30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D2E6C525-4344-462D-A48F-BF1A80500AB8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{D2E6C525-4344-462D-A48F-BF1A80500AB8}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -618,7 +618,16 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{391D1BE4-0BCF-4ED4-8F72-2B4D7E4679F8}" name="Tabella1" displayName="Tabella1" ref="A1:F55" totalsRowShown="0" headerRowDxfId="10" dataDxfId="8" headerRowBorderDxfId="9" tableBorderDxfId="7" totalsRowBorderDxfId="6">
-  <autoFilter ref="A1:F55" xr:uid="{391D1BE4-0BCF-4ED4-8F72-2B4D7E4679F8}"/>
+  <autoFilter ref="A1:F55" xr:uid="{391D1BE4-0BCF-4ED4-8F72-2B4D7E4679F8}">
+    <filterColumn colId="5">
+      <filters>
+        <filter val="1^sem"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F55">
+    <sortCondition ref="C1:C55"/>
+  </sortState>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{E177C9D9-7AD9-4155-A2AD-1B93B3868407}" name="InsegnamentoCourse" dataDxfId="5"/>
     <tableColumn id="2" xr3:uid="{D087D171-9B99-4020-9B8D-EF32EAAFD762}" name="DocenteTeacher" dataDxfId="4"/>
@@ -1000,81 +1009,81 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="C3" s="7">
-        <v>46071</v>
+        <v>46042</v>
       </c>
       <c r="D3" s="8">
         <v>0.58333333333333337</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C4" s="7">
-        <v>46195</v>
+        <v>46043</v>
       </c>
       <c r="D4" s="8">
-        <v>0.58333333333333337</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C5" s="7">
-        <v>46212</v>
+        <v>46043</v>
       </c>
       <c r="D5" s="8">
-        <v>0.58333333333333337</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C6" s="7">
-        <v>46273</v>
+        <v>46045</v>
       </c>
       <c r="D6" s="8">
-        <v>0.58333333333333337</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>44</v>
@@ -1082,179 +1091,179 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C7" s="7">
-        <v>46286</v>
+        <v>46048</v>
       </c>
       <c r="D7" s="8">
         <v>0.58333333333333337</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="C8" s="7">
-        <v>46048</v>
+        <v>46050</v>
       </c>
       <c r="D8" s="8">
-        <v>0.58333333333333337</v>
+        <v>0.60416666666666663</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="C9" s="7">
-        <v>46072</v>
+        <v>46050</v>
       </c>
       <c r="D9" s="8">
-        <v>0.58333333333333337</v>
+        <v>0.60416666666666663</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="C10" s="7">
-        <v>46197</v>
+        <v>46055</v>
       </c>
       <c r="D10" s="8">
         <v>0.375</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="C11" s="7">
-        <v>46231</v>
+        <v>46062</v>
       </c>
       <c r="D11" s="8">
-        <v>0.58333333333333337</v>
+        <v>0.375</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="7">
+        <v>46070</v>
+      </c>
+      <c r="D12" s="8">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="7">
+        <v>46070</v>
+      </c>
+      <c r="D13" s="8">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C14" s="7">
+        <v>46071</v>
+      </c>
+      <c r="D14" s="8">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B15" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="7">
-        <v>46267</v>
-      </c>
-      <c r="D12" s="8">
+      <c r="C15" s="7">
+        <v>46072</v>
+      </c>
+      <c r="D15" s="8">
         <v>0.58333333333333337</v>
       </c>
-      <c r="E12" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F12" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C13" s="7">
-        <v>46287</v>
-      </c>
-      <c r="D13" s="8">
-        <v>0.58333333333333337</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="F13" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C14" s="7">
-        <v>46045</v>
-      </c>
-      <c r="D14" s="8">
-        <v>0.39583333333333331</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="F14" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C15" s="7">
-        <v>46076</v>
-      </c>
-      <c r="D15" s="8">
-        <v>0.39583333333333331</v>
-      </c>
       <c r="E15" s="6" t="s">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>44</v>
@@ -1268,136 +1277,136 @@
         <v>14</v>
       </c>
       <c r="C16" s="7">
-        <v>46189</v>
+        <v>46076</v>
       </c>
       <c r="D16" s="8">
         <v>0.39583333333333331</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="C17" s="7">
-        <v>46209</v>
+        <v>46079</v>
       </c>
       <c r="D17" s="8">
-        <v>0.39583333333333331</v>
+        <v>0.60416666666666663</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="C18" s="7">
-        <v>46272</v>
+        <v>46079</v>
       </c>
       <c r="D18" s="8">
-        <v>0.39583333333333331</v>
+        <v>0.60416666666666663</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>17</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" s="7">
+        <v>46080</v>
+      </c>
+      <c r="D19" s="8">
+        <v>0.375</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C20" s="7">
+        <v>46188</v>
+      </c>
+      <c r="D20" s="8">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B21" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C19" s="7">
-        <v>46288</v>
-      </c>
-      <c r="D19" s="8">
-        <v>0.39583333333333331</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="F19" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C20" s="7">
-        <v>46043</v>
-      </c>
-      <c r="D20" s="8">
-        <v>0.39583333333333331</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>20</v>
-      </c>
       <c r="C21" s="7">
-        <v>46070</v>
+        <v>46189</v>
       </c>
       <c r="D21" s="8">
         <v>0.39583333333333331</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="C22" s="7">
-        <v>46191</v>
+        <v>46190</v>
       </c>
       <c r="D22" s="8">
-        <v>0.39583333333333331</v>
+        <v>0.58333333333333337</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -1408,7 +1417,7 @@
         <v>20</v>
       </c>
       <c r="C23" s="7">
-        <v>46227</v>
+        <v>46191</v>
       </c>
       <c r="D23" s="8">
         <v>0.39583333333333331</v>
@@ -1420,41 +1429,41 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>20</v>
       </c>
       <c r="C24" s="7">
-        <v>46273</v>
+        <v>46191</v>
       </c>
       <c r="D24" s="8">
         <v>0.39583333333333331</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C25" s="7">
-        <v>46288</v>
+        <v>46195</v>
       </c>
       <c r="D25" s="8">
-        <v>0.39583333333333331</v>
+        <v>0.58333333333333337</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>44</v>
@@ -1462,125 +1471,125 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="C26" s="7">
-        <v>46043</v>
+        <v>46197</v>
       </c>
       <c r="D26" s="8">
-        <v>0.39583333333333331</v>
+        <v>0.375</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="C27" s="7">
-        <v>46070</v>
+        <v>46206</v>
       </c>
       <c r="D27" s="8">
-        <v>0.39583333333333331</v>
+        <v>0.60416666666666663</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="C28" s="7">
-        <v>46191</v>
+        <v>46206</v>
       </c>
       <c r="D28" s="8">
-        <v>0.39583333333333331</v>
+        <v>0.60416666666666663</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C29" s="7">
-        <v>46227</v>
+        <v>46209</v>
       </c>
       <c r="D29" s="8">
         <v>0.39583333333333331</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F29" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C30" s="7">
-        <v>46273</v>
+        <v>46212</v>
       </c>
       <c r="D30" s="8">
-        <v>0.39583333333333331</v>
+        <v>0.58333333333333337</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="C31" s="7">
-        <v>46288</v>
+        <v>46213</v>
       </c>
       <c r="D31" s="8">
-        <v>0.39583333333333331</v>
+        <v>0.58333333333333337</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>29</v>
       </c>
@@ -1588,7 +1597,7 @@
         <v>26</v>
       </c>
       <c r="C32" s="7">
-        <v>46050</v>
+        <v>46224</v>
       </c>
       <c r="D32" s="8">
         <v>0.60416666666666663</v>
@@ -1600,121 +1609,121 @@
         <v>45</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C33" s="7">
-        <v>46079</v>
+        <v>46224</v>
       </c>
       <c r="D33" s="8">
         <v>0.60416666666666663</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="C34" s="7">
-        <v>46206</v>
+        <v>46226</v>
       </c>
       <c r="D34" s="8">
-        <v>0.60416666666666663</v>
+        <v>0.58333333333333337</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C35" s="7">
-        <v>46224</v>
+        <v>46227</v>
       </c>
       <c r="D35" s="8">
-        <v>0.60416666666666663</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C36" s="7">
-        <v>46274</v>
+        <v>46227</v>
       </c>
       <c r="D36" s="8">
-        <v>0.60416666666666663</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="F36" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="C37" s="7">
-        <v>46288</v>
+        <v>46231</v>
       </c>
       <c r="D37" s="8">
-        <v>0.60416666666666663</v>
+        <v>0.58333333333333337</v>
       </c>
       <c r="E37" s="6" t="s">
         <v>12</v>
       </c>
       <c r="F37" s="9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C38" s="7">
-        <v>46050</v>
+        <v>46265</v>
       </c>
       <c r="D38" s="8">
-        <v>0.60416666666666663</v>
+        <v>0.375</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>45</v>
@@ -1722,165 +1731,165 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="C39" s="7">
-        <v>46079</v>
+        <v>46267</v>
       </c>
       <c r="D39" s="8">
-        <v>0.60416666666666663</v>
+        <v>0.58333333333333337</v>
       </c>
       <c r="E39" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F39" s="9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C40" s="7">
+        <v>46268</v>
+      </c>
+      <c r="D40" s="8">
+        <v>0.375</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F40" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C41" s="7">
+        <v>46272</v>
+      </c>
+      <c r="D41" s="8">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="E41" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F39" s="9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B40" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C40" s="7">
-        <v>46206</v>
-      </c>
-      <c r="D40" s="8">
-        <v>0.60416666666666663</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="F40" s="9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B41" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C41" s="7">
-        <v>46224</v>
-      </c>
-      <c r="D41" s="8">
-        <v>0.60416666666666663</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>27</v>
-      </c>
       <c r="F41" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="C42" s="7">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="D42" s="8">
-        <v>0.60416666666666663</v>
+        <v>0.58333333333333337</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C43" s="7">
+        <v>46273</v>
+      </c>
+      <c r="D43" s="8">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F43" s="9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C44" s="7">
+        <v>46273</v>
+      </c>
+      <c r="D44" s="8">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F44" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="30" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C45" s="7">
+        <v>46274</v>
+      </c>
+      <c r="D45" s="8">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="E45" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F45" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B43" s="6" t="s">
+      <c r="B46" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C43" s="7">
-        <v>46288</v>
-      </c>
-      <c r="D43" s="8">
+      <c r="C46" s="7">
+        <v>46274</v>
+      </c>
+      <c r="D46" s="8">
         <v>0.60416666666666663</v>
       </c>
-      <c r="E43" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F43" s="9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B44" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C44" s="7">
-        <v>46055</v>
-      </c>
-      <c r="D44" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F44" s="9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B45" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C45" s="7">
-        <v>46080</v>
-      </c>
-      <c r="D45" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="E45" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="F45" s="9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B46" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C46" s="7">
-        <v>46190</v>
-      </c>
-      <c r="D46" s="8">
-        <v>0.58333333333333337</v>
-      </c>
       <c r="E46" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F46" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>32</v>
       </c>
@@ -1888,33 +1897,33 @@
         <v>33</v>
       </c>
       <c r="C47" s="7">
-        <v>46213</v>
+        <v>46280</v>
       </c>
       <c r="D47" s="8">
+        <v>0.375</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F47" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C48" s="7">
+        <v>46282</v>
+      </c>
+      <c r="D48" s="8">
         <v>0.58333333333333337</v>
       </c>
-      <c r="E47" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F47" s="9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B48" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C48" s="7">
-        <v>46265</v>
-      </c>
-      <c r="D48" s="8">
-        <v>0.375</v>
-      </c>
       <c r="E48" s="6" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="F48" s="9" t="s">
         <v>45</v>
@@ -1922,33 +1931,33 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="C49" s="7">
-        <v>46280</v>
+        <v>46286</v>
       </c>
       <c r="D49" s="8">
-        <v>0.375</v>
+        <v>0.58333333333333337</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F49" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="C50" s="7">
-        <v>46042</v>
+        <v>46287</v>
       </c>
       <c r="D50" s="8">
         <v>0.58333333333333337</v>
@@ -1957,104 +1966,104 @@
         <v>13</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="C51" s="7">
-        <v>46062</v>
+        <v>46288</v>
       </c>
       <c r="D51" s="8">
-        <v>0.375</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="C52" s="7">
-        <v>46188</v>
+        <v>46288</v>
       </c>
       <c r="D52" s="8">
-        <v>0.58333333333333337</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="E52" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F52" s="9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C53" s="7">
+        <v>46288</v>
+      </c>
+      <c r="D53" s="8">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="E53" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F53" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="30" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C54" s="7">
+        <v>46288</v>
+      </c>
+      <c r="D54" s="8">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="E54" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F52" s="9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A53" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B53" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C53" s="7">
-        <v>46226</v>
-      </c>
-      <c r="D53" s="8">
-        <v>0.58333333333333337</v>
-      </c>
-      <c r="E53" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="F53" s="9" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B54" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C54" s="7">
-        <v>46268</v>
-      </c>
-      <c r="D54" s="8">
-        <v>0.375</v>
-      </c>
-      <c r="E54" s="6" t="s">
-        <v>34</v>
-      </c>
       <c r="F54" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B55" s="11" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C55" s="12">
-        <v>46282</v>
+        <v>46288</v>
       </c>
       <c r="D55" s="13">
-        <v>0.58333333333333337</v>
+        <v>0.60416666666666663</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>45</v>

</xml_diff>

<commit_message>
Aggiunte nuove mat 2 sem
</commit_message>
<xml_diff>
--- a/segreteria/Calendario esami LM.xlsx
+++ b/segreteria/Calendario esami LM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saint\unipavia\segreteria\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C404D518-2E69-4DC9-BDFD-E76AB847E414}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F63D43B4-2E15-434C-9E7E-F98238FC1CA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D2E6C525-4344-462D-A48F-BF1A80500AB8}"/>
   </bookViews>
@@ -186,7 +186,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -199,6 +199,21 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -321,7 +336,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -365,6 +380,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -630,7 +663,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{391D1BE4-0BCF-4ED4-8F72-2B4D7E4679F8}" name="Tabella1" displayName="Tabella1" ref="A1:G55" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8" totalsRowBorderDxfId="7">
-  <autoFilter ref="A1:G55" xr:uid="{391D1BE4-0BCF-4ED4-8F72-2B4D7E4679F8}"/>
+  <autoFilter ref="A1:G55" xr:uid="{391D1BE4-0BCF-4ED4-8F72-2B4D7E4679F8}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Numerical methods in engineering sciences"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F55">
     <sortCondition ref="C1:C55"/>
   </sortState>
@@ -999,7 +1038,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
@@ -1022,7 +1061,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>35</v>
       </c>
@@ -1045,7 +1084,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>19</v>
       </c>
@@ -1068,7 +1107,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>25</v>
       </c>
@@ -1114,7 +1153,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>8</v>
       </c>
@@ -1137,7 +1176,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>29</v>
       </c>
@@ -1160,7 +1199,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>30</v>
       </c>
@@ -1183,7 +1222,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>32</v>
       </c>
@@ -1206,7 +1245,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>35</v>
       </c>
@@ -1229,7 +1268,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>19</v>
       </c>
@@ -1252,7 +1291,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>25</v>
       </c>
@@ -1275,7 +1314,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>0</v>
       </c>
@@ -1296,7 +1335,7 @@
       </c>
       <c r="G14" s="9"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>8</v>
       </c>
@@ -1320,29 +1359,29 @@
       </c>
     </row>
     <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="7">
+      <c r="C16" s="17">
         <v>46076</v>
       </c>
-      <c r="D16" s="8">
+      <c r="D16" s="18">
         <v>0.39583333333333331</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="F16" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="G16" s="14" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="F16" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="G16" s="20" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>29</v>
       </c>
@@ -1365,7 +1404,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>30</v>
       </c>
@@ -1388,7 +1427,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>32</v>
       </c>
@@ -1411,7 +1450,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>35</v>
       </c>
@@ -1435,29 +1474,29 @@
       </c>
     </row>
     <row r="21" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="C21" s="7">
+      <c r="C21" s="17">
         <v>46189</v>
       </c>
-      <c r="D21" s="8">
+      <c r="D21" s="18">
         <v>0.39583333333333331</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="E21" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="F21" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="G21" s="14" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F21" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="G21" s="20" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>32</v>
       </c>
@@ -1478,7 +1517,7 @@
       </c>
       <c r="G22" s="9"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>19</v>
       </c>
@@ -1501,7 +1540,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>25</v>
       </c>
@@ -1522,7 +1561,7 @@
       </c>
       <c r="G24" s="9"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>0</v>
       </c>
@@ -1543,7 +1582,7 @@
       </c>
       <c r="G25" s="9"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>8</v>
       </c>
@@ -1566,7 +1605,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>29</v>
       </c>
@@ -1589,7 +1628,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>30</v>
       </c>
@@ -1613,29 +1652,29 @@
       </c>
     </row>
     <row r="29" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
+      <c r="A29" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="C29" s="7">
+      <c r="C29" s="17">
         <v>46209</v>
       </c>
-      <c r="D29" s="8">
+      <c r="D29" s="18">
         <v>0.39583333333333331</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="E29" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="F29" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="G29" s="14" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F29" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="G29" s="20" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>0</v>
       </c>
@@ -1658,7 +1697,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>32</v>
       </c>
@@ -1681,7 +1720,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>29</v>
       </c>
@@ -1702,7 +1741,7 @@
       </c>
       <c r="G32" s="9"/>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>30</v>
       </c>
@@ -1723,7 +1762,7 @@
       </c>
       <c r="G33" s="9"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>35</v>
       </c>
@@ -1744,7 +1783,7 @@
       </c>
       <c r="G34" s="9"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>19</v>
       </c>
@@ -1765,7 +1804,7 @@
       </c>
       <c r="G35" s="9"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
         <v>25</v>
       </c>
@@ -1786,7 +1825,7 @@
       </c>
       <c r="G36" s="9"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
         <v>8</v>
       </c>
@@ -1809,7 +1848,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
         <v>32</v>
       </c>
@@ -1830,7 +1869,7 @@
       </c>
       <c r="G38" s="9"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
         <v>8</v>
       </c>
@@ -1853,7 +1892,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
         <v>35</v>
       </c>
@@ -1875,29 +1914,29 @@
       <c r="G40" s="9"/>
     </row>
     <row r="41" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A41" s="5" t="s">
+      <c r="A41" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="B41" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="C41" s="7">
+      <c r="C41" s="17">
         <v>46272</v>
       </c>
-      <c r="D41" s="8">
+      <c r="D41" s="18">
         <v>0.39583333333333331</v>
       </c>
-      <c r="E41" s="6" t="s">
+      <c r="E41" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="F41" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="G41" s="14" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F41" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="G41" s="20" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>0</v>
       </c>
@@ -1918,7 +1957,7 @@
       </c>
       <c r="G42" s="9"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
         <v>19</v>
       </c>
@@ -1941,7 +1980,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
         <v>25</v>
       </c>
@@ -1964,7 +2003,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
         <v>29</v>
       </c>
@@ -1987,7 +2026,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
         <v>30</v>
       </c>
@@ -2008,7 +2047,7 @@
       </c>
       <c r="G46" s="9"/>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>32</v>
       </c>
@@ -2029,7 +2068,7 @@
       </c>
       <c r="G47" s="9"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
         <v>35</v>
       </c>
@@ -2050,7 +2089,7 @@
       </c>
       <c r="G48" s="9"/>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
         <v>0</v>
       </c>
@@ -2071,7 +2110,7 @@
       </c>
       <c r="G49" s="9"/>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
         <v>8</v>
       </c>
@@ -2095,29 +2134,29 @@
       </c>
     </row>
     <row r="51" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A51" s="5" t="s">
+      <c r="A51" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B51" s="6" t="s">
+      <c r="B51" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="C51" s="7">
+      <c r="C51" s="17">
         <v>46288</v>
       </c>
-      <c r="D51" s="8">
+      <c r="D51" s="18">
         <v>0.39583333333333331</v>
       </c>
-      <c r="E51" s="6" t="s">
+      <c r="E51" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="F51" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="G51" s="14" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F51" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="G51" s="20" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
         <v>19</v>
       </c>
@@ -2140,7 +2179,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
         <v>25</v>
       </c>
@@ -2161,7 +2200,7 @@
       </c>
       <c r="G53" s="9"/>
     </row>
-    <row r="54" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
         <v>29</v>
       </c>
@@ -2182,7 +2221,7 @@
       </c>
       <c r="G54" s="9"/>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
         <v>30</v>
       </c>

</xml_diff>